<commit_message>
Changed emails a bit
remote access bruce email and one of the bank emails, and changed replies a bit
</commit_message>
<xml_diff>
--- a/Assets/Editor/EmailDataExample.xlsx
+++ b/Assets/Editor/EmailDataExample.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GameDesign\Programming 3\Final Assignment\Gone Phish\GonePhishing\Assets\Editor\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joshy\Documents\GitHub\GonePhishing\Assets\Editor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9697734C-A269-49A0-831A-91AB6E4681D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E40004A6-02B9-4BB2-ACA1-058A62C95485}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3A1DEF22-8015-43E6-8B07-6E12E7B783C7}"/>
+    <workbookView xWindow="8" yWindow="8" windowWidth="19185" windowHeight="11265" xr2:uid="{3A1DEF22-8015-43E6-8B07-6E12E7B783C7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,9 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -259,9 +262,6 @@
     <t>Hello Admin! Today, there is an uptick of urgent phishing scams, and a general increase in scams that are too good to be true! These are things you might know, like a bunch of free money or a car! Also they could threaten you to accept these fast, so please keep an eye out!</t>
   </si>
   <si>
-    <t>From: Training</t>
-  </si>
-  <si>
     <t>Why do we need this again?</t>
   </si>
   <si>
@@ -287,22 +287,9 @@
     <t>I don’t need you telling me how to do my job, the AI already pesters me.</t>
   </si>
   <si>
-    <t>I’ll keep an eye out.</t>
-  </si>
-  <si>
-    <t>Hello Admin!
-I would like to request all documents related to networking, and server credentials be handed to me through this email. This should be done as soon as you read this email without question.</t>
-  </si>
-  <si>
     <t>Ok, I’ll send them over soon.</t>
   </si>
   <si>
-    <t>Bruce why aren’t you using your email? Is this spam?</t>
-  </si>
-  <si>
-    <t>Who are you?</t>
-  </si>
-  <si>
     <t>D1 2</t>
   </si>
   <si>
@@ -358,12 +345,6 @@
   </si>
   <si>
     <t>Ok Grace, I’ll come by and take a look soon.</t>
-  </si>
-  <si>
-    <t>Grace please punctuate and spell your emails, I don’t know if this is you,</t>
-  </si>
-  <si>
-    <t>I think this is spam.</t>
   </si>
   <si>
     <t>I’m sending this email to you because we’ve had this weird issue recently where the computer we’re using for the audio production locks up and we have to wait like 40 seconds to start using it again. I don’t want any downtime during the times we’re broadcasting, so maybe see about procuring an upgrade for our computer or seeing what’s wrong?
@@ -374,12 +355,6 @@
     <t>I’ll get back to you soon, and I’ll ask management if they can expense it.</t>
   </si>
   <si>
-    <t>I’ll take a look at the computer later.</t>
-  </si>
-  <si>
-    <t>Ivan, you just told me you didn’t need a new computer a few months ago.</t>
-  </si>
-  <si>
     <t>Hey I have this error on my computer that I emailed you about two weeks ago and you ignored me. I emailed last week as well but I didn’t get a reply. I’m getting sick of this, and if you don’t help me, so god help me I’m reporting you to the manager. It’s some pop up saying I’m out of space on my cloud storage, and I can’t save anything!
 MAKE IT GO AWAY!!</t>
   </si>
@@ -387,12 +362,6 @@
     <t>Jeez calm down Jenelle, I’ll take a look now.</t>
   </si>
   <si>
-    <t>Jenelle you sure this is meant for me? Seems super aggressive.</t>
-  </si>
-  <si>
-    <t>This is spam right?</t>
-  </si>
-  <si>
     <t>Yo dude, I got this email from this company, it’s got some sick deals about computers on sale! I think we should take a look actually, it’s like top end hardware for like 99% off! And it’s got a 2 for one deal! What a steal! And it’s not from RamPC! It says we gotta act quick though, the sale only lasts 12 hours. I’m gonna buy some stuff for our department with the company card.</t>
   </si>
   <si>
@@ -490,9 +459,6 @@
   <si>
     <t>From: BruceS@NBC.com
 BRING ME MY CHAIR BACK NOOOOOW</t>
-  </si>
-  <si>
-    <t>Uhh not me.</t>
   </si>
   <si>
     <t>It was grace.</t>
@@ -543,10 +509,6 @@
 -Grace</t>
   </si>
   <si>
-    <t>From: RemoteAccessBruceS@NBO.com_x000D_
-Need Access NOW!</t>
-  </si>
-  <si>
     <t>From: Gully@NBC.com
 Sick PC Deal</t>
   </si>
@@ -592,9 +554,6 @@
 Urgent: Large Sum of Money Spent, Is This You?</t>
   </si>
   <si>
-    <t>You’ve spent over 250,000 thousand dollars today. Are you sure this is you? We’ve locked your card, please contact us if this is you. Otherwise we will call the police on you within 12h.</t>
-  </si>
-  <si>
     <t>From: FinanceDept@NBR.com 
 Urgent: Why did you buy a car</t>
   </si>
@@ -609,6 +568,54 @@
   </si>
   <si>
     <t>They're a fake company. Received an email earlier from them for something else. Keep vigilant on these guys, and maybe try digging deeper?</t>
+  </si>
+  <si>
+    <t>From: Training
+Daily Forecast</t>
+  </si>
+  <si>
+    <t>Ok my bad, I forgot. I'll fix it soon I swear. I'll make it up to you later with a coupon for the local coffee place deal?</t>
+  </si>
+  <si>
+    <t>Sorry for forgetting, I’ll see to it soon. You want me to do anything as an apology?</t>
+  </si>
+  <si>
+    <t>I’ll take a look at the computer later. Let me know if anything else.</t>
+  </si>
+  <si>
+    <t>Ivan, you just told me you didn’t need a new computer a few months ago. I'll still go ask management though, don't worry.</t>
+  </si>
+  <si>
+    <t>Grace please punctuate and spell your emails, I don’t know/can't tell if this is you.</t>
+  </si>
+  <si>
+    <t>Have you tried resetting your password? Also ask the AI to fix your email please, I struggle to read it.</t>
+  </si>
+  <si>
+    <t>Uhh not me. Think it was Jenelle</t>
+  </si>
+  <si>
+    <t>I’ll keep an eye out. Let management know too?</t>
+  </si>
+  <si>
+    <t>Hello Admin, I'm reaching out again for a request. Specifically some documentation for the website backend, management apparently wants to build it up, and contract it off to someone. They need it by the end of the day.</t>
+  </si>
+  <si>
+    <t>I didn't hear nothing about this in your prior email?</t>
+  </si>
+  <si>
+    <t>Bruce why aren’t you using your email? Also this is weird, I could just do it?</t>
+  </si>
+  <si>
+    <t>From: RemoteAccessBruceS@NBO.com
+Need Documention Asap!</t>
+  </si>
+  <si>
+    <t>Hello. This is an automated email notifying you of a large transaction. RAMPC - ASAS 13inch Gaming  Laptop - LTX 7090 InTol 12100S 128GB RAM 
+Total: $4022
+Order Number:091631745 
+This was made by: RemoteAccessBruceS@NBO.Com.
+Let us know if this was you?</t>
   </si>
 </sst>
 </file>
@@ -762,9 +769,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -802,7 +809,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -908,7 +915,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1050,7 +1057,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1059,22 +1066,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4422103-5E59-4D36-B01E-BBBBED35EAD4}">
   <dimension ref="B4:Q30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="4" width="13.5703125" customWidth="1"/>
-    <col min="5" max="5" width="17.5703125" customWidth="1"/>
-    <col min="6" max="6" width="17.42578125" customWidth="1"/>
-    <col min="8" max="10" width="14.5703125" customWidth="1"/>
-    <col min="11" max="11" width="23.5703125" customWidth="1"/>
+    <col min="2" max="4" width="13.59765625" customWidth="1"/>
+    <col min="5" max="5" width="17.59765625" customWidth="1"/>
+    <col min="6" max="6" width="17.3984375" customWidth="1"/>
+    <col min="8" max="10" width="14.59765625" customWidth="1"/>
+    <col min="11" max="11" width="23.59765625" customWidth="1"/>
     <col min="12" max="12" width="48" customWidth="1"/>
-    <col min="13" max="13" width="20.42578125" customWidth="1"/>
-    <col min="14" max="14" width="24.85546875" customWidth="1"/>
-    <col min="15" max="15" width="21.7109375" customWidth="1"/>
-    <col min="16" max="16" width="8.85546875" customWidth="1"/>
-    <col min="17" max="17" width="12.140625" customWidth="1"/>
+    <col min="13" max="13" width="20.3984375" customWidth="1"/>
+    <col min="14" max="14" width="24.86328125" customWidth="1"/>
+    <col min="15" max="15" width="21.73046875" customWidth="1"/>
+    <col min="16" max="16" width="8.86328125" customWidth="1"/>
+    <col min="17" max="17" width="12.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:17" x14ac:dyDescent="0.45">
       <c r="B4" s="2" t="s">
         <v>0</v>
       </c>
@@ -1086,7 +1093,7 @@
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
     </row>
-    <row r="5" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:17" x14ac:dyDescent="0.45">
       <c r="B5" t="s">
         <v>19</v>
       </c>
@@ -1133,7 +1140,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="2:17" ht="90" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:17" ht="71.25" x14ac:dyDescent="0.45">
       <c r="B6" t="s">
         <v>3</v>
       </c>
@@ -1150,29 +1157,29 @@
         <v>5</v>
       </c>
       <c r="H6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I6" t="s">
         <v>72</v>
       </c>
       <c r="J6" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>74</v>
+        <v>171</v>
       </c>
       <c r="L6" s="3" t="s">
         <v>73</v>
       </c>
       <c r="M6" t="s">
+        <v>74</v>
+      </c>
+      <c r="N6" t="s">
         <v>75</v>
       </c>
-      <c r="N6" t="s">
+      <c r="O6" t="s">
         <v>76</v>
       </c>
-      <c r="O6" t="s">
-        <v>77</v>
-      </c>
       <c r="P6" t="s">
         <v>65</v>
       </c>
@@ -1180,7 +1187,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="7" spans="2:17" ht="105" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:17" ht="99.75" x14ac:dyDescent="0.45">
       <c r="B7" t="s">
         <v>20</v>
       </c>
@@ -1197,28 +1204,28 @@
         <v>5</v>
       </c>
       <c r="H7" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="I7" t="s">
         <v>72</v>
       </c>
       <c r="J7" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="K7" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="M7" t="s">
         <v>80</v>
       </c>
-      <c r="L7" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="M7" t="s">
+      <c r="N7" t="s">
         <v>81</v>
       </c>
-      <c r="N7" t="s">
-        <v>82</v>
-      </c>
       <c r="O7" t="s">
-        <v>83</v>
+        <v>179</v>
       </c>
       <c r="P7" t="s">
         <v>65</v>
@@ -1227,7 +1234,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="2:17" ht="120" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:17" ht="99.75" x14ac:dyDescent="0.45">
       <c r="B8" t="s">
         <v>44</v>
       </c>
@@ -1244,28 +1251,28 @@
         <v>55</v>
       </c>
       <c r="H8" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="I8" t="s">
         <v>72</v>
       </c>
       <c r="J8" t="s">
-        <v>161</v>
+        <v>149</v>
       </c>
       <c r="K8" s="3" t="s">
         <v>69</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="M8" t="s">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="N8" t="s">
-        <v>115</v>
+        <v>172</v>
       </c>
       <c r="O8" t="s">
-        <v>116</v>
+        <v>173</v>
       </c>
       <c r="P8" t="s">
         <v>65</v>
@@ -1274,7 +1281,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="9" spans="2:17" ht="135" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:17" ht="128.25" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
         <v>51</v>
       </c>
@@ -1291,28 +1298,28 @@
         <v>54</v>
       </c>
       <c r="H9" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="I9" t="s">
         <v>72</v>
       </c>
       <c r="J9" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="K9" s="3" t="s">
         <v>71</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="M9" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="N9" t="s">
-        <v>111</v>
+        <v>174</v>
       </c>
       <c r="O9" t="s">
-        <v>112</v>
+        <v>175</v>
       </c>
       <c r="P9" t="s">
         <v>65</v>
@@ -1321,7 +1328,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="10" spans="2:17" ht="165" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:17" ht="142.5" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
         <v>47</v>
       </c>
@@ -1338,28 +1345,28 @@
         <v>53</v>
       </c>
       <c r="H10" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="I10" t="s">
         <v>72</v>
       </c>
       <c r="J10" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="K10" s="3" t="s">
         <v>70</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="M10" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="N10" t="s">
-        <v>107</v>
+        <v>176</v>
       </c>
       <c r="O10" t="s">
-        <v>108</v>
+        <v>177</v>
       </c>
       <c r="P10" t="s">
         <v>65</v>
@@ -1368,7 +1375,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="11" spans="2:17" ht="60" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:17" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B11" t="s">
         <v>24</v>
       </c>
@@ -1385,28 +1392,28 @@
         <v>5</v>
       </c>
       <c r="H11" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="I11" t="s">
         <v>72</v>
       </c>
       <c r="J11" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>148</v>
+        <v>137</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>172</v>
+        <v>159</v>
       </c>
       <c r="M11" t="s">
-        <v>149</v>
+        <v>178</v>
       </c>
       <c r="N11" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="O11" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
       <c r="P11" t="s">
         <v>65</v>
@@ -1415,7 +1422,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="2:17" ht="75" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:17" ht="57" x14ac:dyDescent="0.45">
       <c r="B12" t="s">
         <v>25</v>
       </c>
@@ -1432,28 +1439,28 @@
         <v>5</v>
       </c>
       <c r="H12" t="s">
-        <v>126</v>
+        <v>115</v>
       </c>
       <c r="I12" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="J12" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>165</v>
+        <v>183</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>84</v>
+        <v>180</v>
       </c>
       <c r="M12" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="N12" t="s">
-        <v>86</v>
+        <v>182</v>
       </c>
       <c r="O12" t="s">
-        <v>87</v>
+        <v>181</v>
       </c>
       <c r="P12" t="s">
         <v>65</v>
@@ -1462,7 +1469,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="2:17" ht="105" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:17" ht="99.75" x14ac:dyDescent="0.45">
       <c r="B13" t="s">
         <v>22</v>
       </c>
@@ -1479,28 +1486,28 @@
         <v>5</v>
       </c>
       <c r="H13" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="I13" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="J13" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
       <c r="K13" s="3" t="s">
         <v>68</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="M13" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="N13" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="O13" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="P13" t="s">
         <v>65</v>
@@ -1509,7 +1516,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="14" spans="2:17" ht="120" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:17" ht="99.75" x14ac:dyDescent="0.45">
       <c r="B14" t="s">
         <v>62</v>
       </c>
@@ -1526,37 +1533,37 @@
         <v>56</v>
       </c>
       <c r="H14" t="s">
-        <v>128</v>
+        <v>117</v>
       </c>
       <c r="I14" t="s">
         <v>72</v>
       </c>
       <c r="J14" t="s">
-        <v>168</v>
+        <v>155</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>166</v>
+        <v>153</v>
       </c>
       <c r="L14" s="4" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="M14" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="N14" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="O14" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="P14" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
       <c r="Q14" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="15" spans="2:17" ht="60" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:17" ht="57" x14ac:dyDescent="0.45">
       <c r="B15" t="s">
         <v>57</v>
       </c>
@@ -1573,28 +1580,28 @@
         <v>56</v>
       </c>
       <c r="H15" t="s">
-        <v>129</v>
+        <v>118</v>
       </c>
       <c r="I15" t="s">
         <v>72</v>
       </c>
       <c r="J15" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="K15" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="L15" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="M15" t="s">
+        <v>96</v>
+      </c>
+      <c r="N15" t="s">
         <v>163</v>
       </c>
-      <c r="L15" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="M15" t="s">
-        <v>101</v>
-      </c>
-      <c r="N15" t="s">
-        <v>176</v>
-      </c>
       <c r="O15" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="P15" t="s">
         <v>65</v>
@@ -1603,7 +1610,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="16" spans="2:17" ht="225" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:17" ht="199.5" x14ac:dyDescent="0.45">
       <c r="B16" t="s">
         <v>6</v>
       </c>
@@ -1620,13 +1627,13 @@
         <v>18</v>
       </c>
       <c r="H16" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
       <c r="I16" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="J16" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
       <c r="K16" s="3" t="s">
         <v>67</v>
@@ -1635,13 +1642,13 @@
         <v>66</v>
       </c>
       <c r="M16" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="N16" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="O16" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="P16" t="s">
         <v>65</v>
@@ -1650,95 +1657,95 @@
         <v>65</v>
       </c>
     </row>
-    <row r="17" spans="5:17" ht="75" x14ac:dyDescent="0.25">
+    <row r="17" spans="5:17" ht="99.75" x14ac:dyDescent="0.45">
       <c r="E17" s="1"/>
       <c r="H17" t="s">
-        <v>131</v>
+        <v>120</v>
       </c>
       <c r="I17" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="J17" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>178</v>
+        <v>165</v>
       </c>
       <c r="L17" s="4" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="M17" t="s">
+        <v>110</v>
+      </c>
+      <c r="N17" t="s">
+        <v>111</v>
+      </c>
+      <c r="O17" t="s">
+        <v>112</v>
+      </c>
+      <c r="P17" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="18" spans="5:17" ht="57" x14ac:dyDescent="0.45">
+      <c r="H18" t="s">
         <v>121</v>
       </c>
-      <c r="N17" t="s">
+      <c r="I18" t="s">
+        <v>85</v>
+      </c>
+      <c r="J18" t="s">
+        <v>147</v>
+      </c>
+      <c r="K18" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="L18" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="M18" t="s">
+        <v>113</v>
+      </c>
+      <c r="N18" t="s">
+        <v>114</v>
+      </c>
+      <c r="O18" t="s">
+        <v>164</v>
+      </c>
+      <c r="P18" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="19" spans="5:17" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="H19" s="3" t="s">
         <v>122</v>
-      </c>
-      <c r="O17" t="s">
-        <v>123</v>
-      </c>
-      <c r="P17" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q17" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="18" spans="5:17" ht="75" x14ac:dyDescent="0.25">
-      <c r="H18" t="s">
-        <v>132</v>
-      </c>
-      <c r="I18" t="s">
-        <v>90</v>
-      </c>
-      <c r="J18" t="s">
-        <v>159</v>
-      </c>
-      <c r="K18" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="L18" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="M18" t="s">
-        <v>124</v>
-      </c>
-      <c r="N18" t="s">
-        <v>125</v>
-      </c>
-      <c r="O18" t="s">
-        <v>177</v>
-      </c>
-      <c r="P18" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q18" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="19" spans="5:17" ht="45" x14ac:dyDescent="0.25">
-      <c r="H19" s="3" t="s">
-        <v>133</v>
       </c>
       <c r="I19" s="3" t="s">
         <v>72</v>
       </c>
       <c r="J19" t="s">
-        <v>168</v>
+        <v>155</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="N19" s="3" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="O19" s="3" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="P19" t="s">
         <v>65</v>
@@ -1747,30 +1754,30 @@
         <v>65</v>
       </c>
     </row>
-    <row r="20" spans="5:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="5:17" ht="28.5" x14ac:dyDescent="0.45">
       <c r="H20" s="3" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="I20" s="3" t="s">
         <v>72</v>
       </c>
       <c r="J20" t="s">
-        <v>168</v>
+        <v>155</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="M20" t="s">
-        <v>143</v>
+        <v>132</v>
       </c>
       <c r="N20" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="O20" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="P20" t="s">
         <v>65</v>
@@ -1779,30 +1786,30 @@
         <v>65</v>
       </c>
     </row>
-    <row r="21" spans="5:17" ht="195" x14ac:dyDescent="0.25">
+    <row r="21" spans="5:17" ht="171" x14ac:dyDescent="0.45">
       <c r="H21" s="3" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
       <c r="I21" s="3" t="s">
         <v>72</v>
       </c>
       <c r="J21" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>175</v>
+        <v>162</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="M21" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="N21" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="O21" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
       <c r="P21" t="s">
         <v>65</v>
@@ -1811,30 +1818,30 @@
         <v>65</v>
       </c>
     </row>
-    <row r="22" spans="5:17" ht="105" x14ac:dyDescent="0.25">
+    <row r="22" spans="5:17" ht="99.75" x14ac:dyDescent="0.45">
       <c r="H22" s="3" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="I22" s="3" t="s">
         <v>72</v>
       </c>
       <c r="J22" t="s">
+        <v>149</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="L22" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="K22" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="L22" s="3" t="s">
-        <v>174</v>
-      </c>
       <c r="M22" t="s">
-        <v>182</v>
+        <v>168</v>
       </c>
       <c r="N22" t="s">
-        <v>184</v>
+        <v>170</v>
       </c>
       <c r="O22" t="s">
-        <v>183</v>
+        <v>169</v>
       </c>
       <c r="P22" t="s">
         <v>65</v>
@@ -1843,30 +1850,30 @@
         <v>65</v>
       </c>
     </row>
-    <row r="23" spans="5:17" ht="135" x14ac:dyDescent="0.25">
+    <row r="23" spans="5:17" ht="114" x14ac:dyDescent="0.45">
       <c r="H23" s="3" t="s">
-        <v>171</v>
+        <v>158</v>
       </c>
       <c r="I23" s="3" t="s">
         <v>72</v>
       </c>
       <c r="J23" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>169</v>
+        <v>156</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>170</v>
+        <v>157</v>
       </c>
       <c r="N23" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="O23" s="3" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="P23" t="s">
         <v>65</v>
@@ -1875,7 +1882,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="24" spans="5:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="24" spans="5:17" ht="28.5" x14ac:dyDescent="0.45">
       <c r="H24" s="3"/>
       <c r="I24" s="3"/>
       <c r="J24" t="s">
@@ -1891,7 +1898,7 @@
       <c r="P24" s="3"/>
       <c r="Q24" s="3"/>
     </row>
-    <row r="25" spans="5:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="25" spans="5:17" ht="28.5" x14ac:dyDescent="0.45">
       <c r="H25" s="3"/>
       <c r="I25" s="3"/>
       <c r="J25" t="s">
@@ -1907,7 +1914,7 @@
       <c r="P25" s="3"/>
       <c r="Q25" s="3"/>
     </row>
-    <row r="26" spans="5:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="26" spans="5:17" ht="28.5" x14ac:dyDescent="0.45">
       <c r="H26" s="3"/>
       <c r="I26" s="3"/>
       <c r="J26" t="s">
@@ -1923,7 +1930,7 @@
       <c r="P26" s="3"/>
       <c r="Q26" s="3"/>
     </row>
-    <row r="27" spans="5:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="5:17" ht="28.5" x14ac:dyDescent="0.45">
       <c r="H27" s="3"/>
       <c r="I27" s="3"/>
       <c r="J27" s="3"/>
@@ -1937,7 +1944,7 @@
       <c r="P27" s="3"/>
       <c r="Q27" s="3"/>
     </row>
-    <row r="28" spans="5:17" ht="30" x14ac:dyDescent="0.25">
+    <row r="28" spans="5:17" ht="28.5" x14ac:dyDescent="0.45">
       <c r="H28" s="3"/>
       <c r="I28" s="3"/>
       <c r="J28" s="3"/>
@@ -1951,7 +1958,7 @@
       <c r="P28" s="3"/>
       <c r="Q28" s="3"/>
     </row>
-    <row r="29" spans="5:17" x14ac:dyDescent="0.25">
+    <row r="29" spans="5:17" x14ac:dyDescent="0.45">
       <c r="H29" s="3"/>
       <c r="I29" s="3"/>
       <c r="J29" s="3"/>
@@ -1963,7 +1970,7 @@
       <c r="P29" s="3"/>
       <c r="Q29" s="3"/>
     </row>
-    <row r="30" spans="5:17" x14ac:dyDescent="0.25">
+    <row r="30" spans="5:17" x14ac:dyDescent="0.45">
       <c r="H30" s="3"/>
       <c r="I30" s="3"/>
       <c r="J30" s="3"/>

</xml_diff>

<commit_message>
Emails Updated for modern story
</commit_message>
<xml_diff>
--- a/Assets/Editor/EmailDataExample.xlsx
+++ b/Assets/Editor/EmailDataExample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joshy\Documents\GitHub\GonePhishing\Assets\Editor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E40004A6-02B9-4BB2-ACA1-058A62C95485}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEC38ECB-3312-45FA-90E1-F3FA1AD31FCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8" yWindow="8" windowWidth="19185" windowHeight="11265" xr2:uid="{3A1DEF22-8015-43E6-8B07-6E12E7B783C7}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="179">
   <si>
     <t>Sender</t>
   </si>
@@ -226,70 +226,21 @@
   </si>
   <si>
     <t>Hi</t>
-  </si>
-  <si>
-    <t>Hello we were wondering if you would be interested in having a locally owned bakery come onto your show. We are willing to supply the crew with free pastries and bread during shooting. You will find our business info and menu attached in this email. Hope to hear from you soon and let us know if you are interested in this partnership.
-Regards,
-Head Chef Mary
-Attachments:
-Menu.pdf
-BaggyBaguettesInfo.exe</t>
-  </si>
-  <si>
-    <t>From: Baggybaguettes@gmail.com
-Bakery On The News?</t>
-  </si>
-  <si>
-    <t>From: Hiring@NRB.com
-Job Offer</t>
-  </si>
-  <si>
-    <t>From: Jenelle@NBC.com  
-Stupid IT! Fix this now!!!</t>
   </si>
   <si>
     <t>From: Grace@NBC.com 
 hlep me</t>
   </si>
   <si>
-    <t>From: Ivan@NBC.com 
-Need some assistance</t>
-  </si>
-  <si>
     <t>No</t>
   </si>
   <si>
     <t>Hello Admin! Today, there is an uptick of urgent phishing scams, and a general increase in scams that are too good to be true! These are things you might know, like a bunch of free money or a car! Also they could threaten you to accept these fast, so please keep an eye out!</t>
   </si>
   <si>
-    <t>Why do we need this again?</t>
-  </si>
-  <si>
-    <t>Piss Off!</t>
-  </si>
-  <si>
-    <t>Thank You!</t>
-  </si>
-  <si>
     <t>D1 1</t>
   </si>
   <si>
-    <t>Hello admin, I hope you’re doing well. Recently, our company has been under some intense public scrutiny due to some… ethical concerns. As a result, some internet sleuths may be trying to breach the system. Keep an eye out for anything suspicious, like something needing to get done now, or anything that seems too good to be true. Good luck.</t>
-  </si>
-  <si>
-    <t>From: BruceS@NBC.com
-Heads Up!</t>
-  </si>
-  <si>
-    <t>Ok, thank you!</t>
-  </si>
-  <si>
-    <t>I don’t need you telling me how to do my job, the AI already pesters me.</t>
-  </si>
-  <si>
-    <t>Ok, I’ll send them over soon.</t>
-  </si>
-  <si>
     <t>D1 2</t>
   </si>
   <si>
@@ -302,93 +253,15 @@
     <t>D1 4</t>
   </si>
   <si>
-    <t>Good day we are looking to buy your skills from our competitors and are willing to offer 120k as your starting salary, and a signing bonus of 30k. If this interest you in quitting your job then have a look at the contract attached to this email and come down to our location. We need a response within 48h, or we WILL move on with a different candidate.</t>
-  </si>
-  <si>
-    <t>Ok, I’ll look at it and reply soon!</t>
-  </si>
-  <si>
-    <t>Can I get more info?</t>
-  </si>
-  <si>
-    <t>I didn’t apply for no job recently?</t>
-  </si>
-  <si>
-    <t>No one does business for free.</t>
-  </si>
-  <si>
-    <t>Sounds great! We’ll let you know more later.</t>
-  </si>
-  <si>
-    <t>I’m not sure if this is spam or what, please email back if not.</t>
-  </si>
-  <si>
     <t>D1 5</t>
   </si>
   <si>
     <t>D1 6</t>
   </si>
   <si>
-    <t>Can’t say I do, though I did just get an email asking for some employee info.</t>
-  </si>
-  <si>
-    <t>Jenelle might know, she does get around more than us.</t>
-  </si>
-  <si>
-    <t>Before I clock out for the day, I’ve been checking the status on the cameras cause the system keeps flagging an unauthorized connection. Problem is, it won’t tell more details and I can’t do anything with out this dumb company we hired to send someone to come look at it so our contract doesn’t break. This is dumb as hell, and it’s just cause we wanted to save money. Just don’t relay on the cameras to capture everything for awhile.</t>
-  </si>
-  <si>
-    <t>Gotcha, I’ll keep note of it. Probably going to send an email to everyone as well.</t>
-  </si>
-  <si>
-    <t>Let me take a look then I’ll ask the contractor. Likely will send an email letting everyone know tom as well.</t>
-  </si>
-  <si>
     <t>Ok Grace, I’ll come by and take a look soon.</t>
   </si>
   <si>
-    <t>I’m sending this email to you because we’ve had this weird issue recently where the computer we’re using for the audio production locks up and we have to wait like 40 seconds to start using it again. I don’t want any downtime during the times we’re broadcasting, so maybe see about procuring an upgrade for our computer or seeing what’s wrong?
-Kindly,
-Ivan</t>
-  </si>
-  <si>
-    <t>I’ll get back to you soon, and I’ll ask management if they can expense it.</t>
-  </si>
-  <si>
-    <t>Hey I have this error on my computer that I emailed you about two weeks ago and you ignored me. I emailed last week as well but I didn’t get a reply. I’m getting sick of this, and if you don’t help me, so god help me I’m reporting you to the manager. It’s some pop up saying I’m out of space on my cloud storage, and I can’t save anything!
-MAKE IT GO AWAY!!</t>
-  </si>
-  <si>
-    <t>Jeez calm down Jenelle, I’ll take a look now.</t>
-  </si>
-  <si>
-    <t>Yo dude, I got this email from this company, it’s got some sick deals about computers on sale! I think we should take a look actually, it’s like top end hardware for like 99% off! And it’s got a 2 for one deal! What a steal! And it’s not from RamPC! It says we gotta act quick though, the sale only lasts 12 hours. I’m gonna buy some stuff for our department with the company card.</t>
-  </si>
-  <si>
-    <t>Gully, this seems way too good to be true, don’t buy anything.</t>
-  </si>
-  <si>
-    <t>Hang on, take a look at RamPC and see if they’re legit, then buy it.</t>
-  </si>
-  <si>
-    <t>Sounds good, let me know how it goes!</t>
-  </si>
-  <si>
-    <t>I think one of our coworkers just fell for a phishing scam.</t>
-  </si>
-  <si>
-    <t>This isn’t real.</t>
-  </si>
-  <si>
-    <t>This is not us, find someone else.</t>
-  </si>
-  <si>
-    <t>I think your files are wrong or messed up cause I never bought a car.</t>
-  </si>
-  <si>
-    <t>Ask Bruce, looks like something he’d buy, not me.</t>
-  </si>
-  <si>
     <t>D1 7</t>
   </si>
   <si>
@@ -416,9 +289,6 @@
     <t>G1 Bad</t>
   </si>
   <si>
-    <t>Suspicious Attatchments</t>
-  </si>
-  <si>
     <t>Oh dude for real? Thank god I didn’t put anything in yet. That coulda been bad coulda gotten fired or something!</t>
   </si>
   <si>
@@ -431,14 +301,6 @@
     <t>Hoolly shit, thank god you listened to me.</t>
   </si>
   <si>
-    <t>From: Gully@NBC.com
-That would have been dumb</t>
-  </si>
-  <si>
-    <t>From: Gully@NBC.com
-Its over bro</t>
-  </si>
-  <si>
     <t>Oh shit dude, I think I fell for a scam… I’m done for..</t>
   </si>
   <si>
@@ -457,37 +319,12 @@
     <t>D1 14</t>
   </si>
   <si>
-    <t>From: BruceS@NBC.com
-BRING ME MY CHAIR BACK NOOOOOW</t>
-  </si>
-  <si>
-    <t>It was grace.</t>
-  </si>
-  <si>
-    <t>It was Ivan.</t>
-  </si>
-  <si>
-    <t>Just got word from a old place I worked at that they had to shut down the company due to a bunch of files being leaked. A bunch of people just lost there jobs due to some annoying person who decide to get there hands on files and leak them to the world. Goes to show you just how much of a danger these people are. Apparently some hacker from another company managed to get into their systems due to a tech manager opening a email and clicking a link that installed malware. From there they leaked everything to the company that hired them. We gotta be aware of stuff like this, we can’t be running into the same crap.</t>
-  </si>
-  <si>
-    <t>Agreed, the world is a scary place and we gotta keep vigilant.</t>
-  </si>
-  <si>
-    <t>Keep me posted on this, that’s something to watch over the next while.</t>
-  </si>
-  <si>
-    <t>Certainly interesting, we gotta keep our eyes peeled for stuff like this for sure.</t>
-  </si>
-  <si>
     <t>g1</t>
   </si>
   <si>
     <t>AI Phishing Assistant</t>
   </si>
   <si>
-    <t>Bruce</t>
-  </si>
-  <si>
     <t>Hacker</t>
   </si>
   <si>
@@ -500,122 +337,255 @@
     <t>Grace</t>
   </si>
   <si>
-    <t>From: Ivan@NBC.com 
-Gift Card Scam?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Hi dear, i need a new phone my one is freezing all the time. I download this app and it start lagging my phone. It asks for login information to but i dont know what to put in can you help me please. Also i got this email from you guys. It asked about a subscription but i dont remember a subscription. Help me cancel it too please. 
--Grace</t>
-  </si>
-  <si>
-    <t>From: Gully@NBC.com
-Sick PC Deal</t>
-  </si>
-  <si>
     <t>Looping in everyone here, just got an email asking about a free gift card, can’t say I recall any raffles around here? Maybe I don’t go outside enough(or socialize) though, and one of you know about this?</t>
   </si>
   <si>
     <t>Gully</t>
   </si>
   <si>
-    <t>From: Ivan@NBC.com 
-Mysterious Camera Connection</t>
-  </si>
-  <si>
-    <t>Hmm, I’ll take a look tomorrow.  Think I’ll send an email companywide as well.</t>
-  </si>
-  <si>
     <t>D1 16</t>
-  </si>
-  <si>
-    <t>TO ALL EMPLOYEES 
-WHO THE HELL STOLE MY CHAIR FROM MY OFFICE. REPLY NOW OR I WILL FIND YOU AND BREAK YOUR CHAIR!</t>
-  </si>
-  <si>
-    <t>From: Jenelle@NBC.com
-Offer Code Legit?</t>
-  </si>
-  <si>
-    <t>Hi Admin, thanks for *finally* listening to me and my problems, I expect this error to go away soon right? Anyway, I'm emailing for a 48h offer code we got from these guys, called Baggy Baggutes. They seem legit but hard to know. Can you verify this for me? I did some digging but the spot seems local, unless the website was fake or something</t>
-  </si>
-  <si>
-    <t>From: Ivan@NBC.com
-Seedy World</t>
-  </si>
-  <si>
-    <t>No, not sure about that one, Maybe Grace knows, she’s a real penny pincher.</t>
-  </si>
-  <si>
-    <t>Find someone else, I’m too broke for a Grotti.</t>
-  </si>
-  <si>
-    <t>From: NovaBank@Notify.com 
-Urgent: Large Sum of Money Spent, Is This You?</t>
-  </si>
-  <si>
-    <t>From: FinanceDept@NBR.com 
-Urgent: Why did you buy a car</t>
-  </si>
-  <si>
-    <t>I am writing to you as we have on your files that a 100,000 car from Grotti was bought in your name and you have not paid any taxes for this. Let us know ASAP if this is you, otherwise we will pursue legal action.</t>
-  </si>
-  <si>
-    <t>Just got an email from them, they're fake.</t>
-  </si>
-  <si>
-    <t>Think they're legit, should be good.</t>
-  </si>
-  <si>
-    <t>They're a fake company. Received an email earlier from them for something else. Keep vigilant on these guys, and maybe try digging deeper?</t>
   </si>
   <si>
     <t>From: Training
 Daily Forecast</t>
   </si>
   <si>
-    <t>Ok my bad, I forgot. I'll fix it soon I swear. I'll make it up to you later with a coupon for the local coffee place deal?</t>
-  </si>
-  <si>
-    <t>Sorry for forgetting, I’ll see to it soon. You want me to do anything as an apology?</t>
-  </si>
-  <si>
-    <t>I’ll take a look at the computer later. Let me know if anything else.</t>
-  </si>
-  <si>
-    <t>Ivan, you just told me you didn’t need a new computer a few months ago. I'll still go ask management though, don't worry.</t>
-  </si>
-  <si>
-    <t>Grace please punctuate and spell your emails, I don’t know/can't tell if this is you.</t>
-  </si>
-  <si>
-    <t>Have you tried resetting your password? Also ask the AI to fix your email please, I struggle to read it.</t>
-  </si>
-  <si>
-    <t>Uhh not me. Think it was Jenelle</t>
-  </si>
-  <si>
     <t>I’ll keep an eye out. Let management know too?</t>
   </si>
   <si>
-    <t>Hello Admin, I'm reaching out again for a request. Specifically some documentation for the website backend, management apparently wants to build it up, and contract it off to someone. They need it by the end of the day.</t>
-  </si>
-  <si>
-    <t>I didn't hear nothing about this in your prior email?</t>
-  </si>
-  <si>
-    <t>Bruce why aren’t you using your email? Also this is weird, I could just do it?</t>
-  </si>
-  <si>
-    <t>From: RemoteAccessBruceS@NBO.com
-Need Documention Asap!</t>
-  </si>
-  <si>
-    <t>Hello. This is an automated email notifying you of a large transaction. RAMPC - ASAS 13inch Gaming  Laptop - LTX 7090 InTol 12100S 128GB RAM 
-Total: $4022
-Order Number:091631745 
-This was made by: RemoteAccessBruceS@NBO.Com.
-Let us know if this was you?</t>
+    <t>From: SP@XCEL.com
+Welcome!</t>
+  </si>
+  <si>
+    <t>Hey so you’re the new admin huh? The team here has been waiting on one for a while, so please do us good! Let us know if anything!
+-Ivan, Jenelle, Grace, Selina, Gully</t>
+  </si>
+  <si>
+    <t>Ok!</t>
+  </si>
+  <si>
+    <t>This seems to be automated.</t>
+  </si>
+  <si>
+    <t>Maybe someone will tell me what this is later?</t>
+  </si>
+  <si>
+    <t>Hello Admin! I am a supervisor overseeing your first day here. Welcome to your first day at XCEL, the place where you’ll excel in all aspects and go further than ever before! Please ignore the AI message earlier, we haven't had a chance to wipe the computer. We’ve put you in a virtual environment as per company policy, and want you to answer these emails for us, for your first day.</t>
+  </si>
+  <si>
+    <t>Will do!</t>
+  </si>
+  <si>
+    <t>I hope the emails aren't too important…</t>
+  </si>
+  <si>
+    <t>Thank you guys!</t>
+  </si>
+  <si>
+    <t>I'll try my best!</t>
+  </si>
+  <si>
+    <t>I'll let you know if anything, don't worry!</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>Supervisor</t>
+  </si>
+  <si>
+    <t>From: Ivan@XCEL.com  
+Welcome to the team!</t>
+  </si>
+  <si>
+    <t>From: SP@XCEL.com 
+One More Thing!</t>
+  </si>
+  <si>
+    <t>Oh one more thing! You are in charge of manually filtering all emails sent to your team, so please be aware they may be of high importance to said team!</t>
+  </si>
+  <si>
+    <t>So much for emails being unimportant…</t>
+  </si>
+  <si>
+    <t>Sounds good!</t>
+  </si>
+  <si>
+    <t>Talk about a workload…</t>
+  </si>
+  <si>
+    <t>Microsoft 365 is holding all further communications, please verify your identity by simply replying with your email. This is a new verification method we are trialing at your company. After replying, all communications will be released.</t>
+  </si>
+  <si>
+    <t>From: M365Security@Microsoft.com 
+URGENT! Email Hold</t>
+  </si>
+  <si>
+    <t>First time seeing this, Admin@XCEL.net</t>
+  </si>
+  <si>
+    <t>Admin@XCEL.net</t>
+  </si>
+  <si>
+    <t>Now that’s pretty high tech: Admin@XCEL.net</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hey Admin, it’s me Jenelle. I gotta say, not great first terms, cause I got an email from you asking for my account info, and I gave it to you(and the two factor code). Afterward I saw a remote request, and accepted it. Then I see that hacking terminal thing pop up and my computer shuts down. Then next thing I know, I hear Grace and Ivan saying they got the same email from you. I think whoever sent you an email got your identity and started passing it around to hack the team. </t>
+  </si>
+  <si>
+    <t>From: Jenelle@XCEL.com
+This can't be you?</t>
+  </si>
+  <si>
+    <t>That wasn’t me, contact IT now!!!</t>
+  </si>
+  <si>
+    <t>Oh ssshit.</t>
+  </si>
+  <si>
+    <t>Jenelle tell them to not reply, I screwed up big time.</t>
+  </si>
+  <si>
+    <t>Hey sorry for that email just now, we’re testing an AI filter to get rid of this menial work but looks like it got some emails through. Keep your eyes peeled.</t>
+  </si>
+  <si>
+    <t>From: SP@XCEL.com
+My bad!</t>
+  </si>
+  <si>
+    <t>Could of told me that before!</t>
+  </si>
+  <si>
+    <t>Should make sure that works beforehand.</t>
+  </si>
+  <si>
+    <t>Good to know.</t>
+  </si>
+  <si>
+    <t>From: Gully@XCEL.com
+Sick PC Deal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yo Admin, good meeting you! I got this email from this company, it’s got some sick deals about computers on sale! I think we should take a look actually, it’s like top end hardware for like 75% off! And it’s got a 2 for one deal! What a steal! And it’s not from TEMU! It says we gotta act quick though, the sale only lasts 12 hours. I’m gonna buy some stuff for our department with the company card. </t>
+  </si>
+  <si>
+    <t>All right Gully, let me know how it goes!</t>
+  </si>
+  <si>
+    <t>TEMU got some good stuff though! Regardless the deal looks legit.</t>
+  </si>
+  <si>
+    <t>Looks legit, place an order!</t>
+  </si>
+  <si>
+    <t>*THIS MESSAGE MUST BE FILTERED BEFORE BEING SENT
+Hey, hope you’re well! Just emailing about this gathering we wanted to host, and whether or not you’re interested. Download this file for more details please!
+inv.msi</t>
+  </si>
+  <si>
+    <t>From: JM@Gmail.com
+RSVP</t>
+  </si>
+  <si>
+    <t>Seems legit, I’ll forward it to her.</t>
+  </si>
+  <si>
+    <t>Ms. Popular over here, can’t deny this from her.</t>
+  </si>
+  <si>
+    <t>This is what they meant by manual filtering… Still gotta send it to her though.</t>
+  </si>
+  <si>
+    <t>Jenelle or Selina might know, they do get around more than us.</t>
+  </si>
+  <si>
+    <t>No, not sure about that one, Maybe Grace or Gully knows, they're real penny pinchers.</t>
+  </si>
+  <si>
+    <t>Can’t say I do. Too broke to shop lol</t>
+  </si>
+  <si>
+    <t>From: Google-Flagging-System@Gmail.com</t>
+  </si>
+  <si>
+    <t>Log in and verify the sign in was someone from IT.</t>
+  </si>
+  <si>
+    <t>Log in and change password.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Log in and reset everything. </t>
+  </si>
+  <si>
+    <t>An unidentified sign in was detected. If this is you, you can ignore it. If not, please use the link below and log into your google account to change your password within 12h, or your account will be closed.</t>
+  </si>
+  <si>
+    <t>Grace, your email is a bit hard to read, can you run a spellcheck on it next time?</t>
+  </si>
+  <si>
+    <t>Hi dear, i need a new phone my one is freezing all the time. I download this app and it start lagging my phone. It asks for login information to but i dont know what to put in can you help me please. Also I want to know if there's any discounts for uber, do you know if the company has any?</t>
+  </si>
+  <si>
+    <t>Try turning it off and on again?cAlso ask Ivan about the discounts, I just got here.</t>
+  </si>
+  <si>
+    <t>From: Grace@XCEL.com
+help me</t>
+  </si>
+  <si>
+    <t>From: Selina@XCEL.com
+Help Needed Tommorow!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Good day Admin, my mom died recently, and I’ve been struggling to make ends meet. I was thinking about setting up a gofundme to offset some of the funeral costs. I know you're new and all, but Ivan and Gully are too busy to set it up, so can you help me?
+</t>
+  </si>
+  <si>
+    <t>For sure!</t>
+  </si>
+  <si>
+    <t>Send me your info for the listing tommorow, and I’ll set up the gofundme, hopefully it goes well!</t>
+  </si>
+  <si>
+    <t>They can't be that busy right? Regardless I'll help you out, no worries.</t>
+  </si>
+  <si>
+    <t>Selina</t>
+  </si>
+  <si>
+    <t>From: Ivan@XCEL.com 
+Gift Card Scam?</t>
+  </si>
+  <si>
+    <t>From: Gully@XCEL.com
+That would have been dumb</t>
+  </si>
+  <si>
+    <t>From: Gully@XCEL.com
+Its over bro</t>
+  </si>
+  <si>
+    <t>From: SP@XCEL.com
+Its over bro</t>
+  </si>
+  <si>
+    <t>Tough test!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">You have done well today based on the phishing emails you managed to complete. Most emails we tested on you, but some we left out and even our team was stumped on some, so don't feel bad about missing them(if you did). Please convene with your team tommorow about the results, as their emails were real, and whatever they needed from you, you'll have to do. </t>
+  </si>
+  <si>
+    <t>Wow, what a day. And I will let my team know, thanks.</t>
+  </si>
+  <si>
+    <t>Make them easier please! Also, will do on the team stuff, thanks for the reminder.</t>
+  </si>
+  <si>
+    <t>Impersonation/fill in whatever</t>
+  </si>
+  <si>
+    <t>Np</t>
   </si>
 </sst>
 </file>
@@ -683,7 +653,34 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="6">
+    <dxf>
+      <border>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
     <dxf>
       <border>
         <top style="thin">
@@ -1157,28 +1154,28 @@
         <v>5</v>
       </c>
       <c r="H6" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="I6" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="J6" t="s">
-        <v>145</v>
+        <v>97</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>171</v>
+        <v>105</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="M6" t="s">
-        <v>74</v>
+        <v>109</v>
       </c>
       <c r="N6" t="s">
-        <v>75</v>
+        <v>110</v>
       </c>
       <c r="O6" t="s">
-        <v>76</v>
+        <v>111</v>
       </c>
       <c r="P6" t="s">
         <v>65</v>
@@ -1204,28 +1201,28 @@
         <v>5</v>
       </c>
       <c r="H7" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="I7" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="J7" t="s">
-        <v>146</v>
+        <v>119</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="M7" t="s">
-        <v>80</v>
+        <v>113</v>
       </c>
       <c r="N7" t="s">
-        <v>81</v>
+        <v>114</v>
       </c>
       <c r="O7" t="s">
-        <v>179</v>
+        <v>106</v>
       </c>
       <c r="P7" t="s">
         <v>65</v>
@@ -1234,7 +1231,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="2:17" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:17" ht="71.25" x14ac:dyDescent="0.45">
       <c r="B8" t="s">
         <v>44</v>
       </c>
@@ -1251,28 +1248,28 @@
         <v>55</v>
       </c>
       <c r="H8" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="I8" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="J8" t="s">
-        <v>149</v>
+        <v>118</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>69</v>
+        <v>120</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="M8" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="N8" t="s">
-        <v>172</v>
+        <v>116</v>
       </c>
       <c r="O8" t="s">
-        <v>173</v>
+        <v>117</v>
       </c>
       <c r="P8" t="s">
         <v>65</v>
@@ -1281,7 +1278,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="9" spans="2:17" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:17" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
         <v>51</v>
       </c>
@@ -1298,28 +1295,28 @@
         <v>54</v>
       </c>
       <c r="H9" t="s">
-        <v>86</v>
+        <v>73</v>
       </c>
       <c r="I9" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="J9" t="s">
-        <v>148</v>
+        <v>99</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>71</v>
+        <v>121</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>102</v>
+        <v>122</v>
       </c>
       <c r="M9" t="s">
-        <v>103</v>
+        <v>123</v>
       </c>
       <c r="N9" t="s">
-        <v>174</v>
+        <v>124</v>
       </c>
       <c r="O9" t="s">
-        <v>175</v>
+        <v>125</v>
       </c>
       <c r="P9" t="s">
         <v>65</v>
@@ -1328,7 +1325,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="10" spans="2:17" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:17" ht="71.25" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
         <v>47</v>
       </c>
@@ -1345,28 +1342,28 @@
         <v>53</v>
       </c>
       <c r="H10" t="s">
-        <v>94</v>
+        <v>74</v>
       </c>
       <c r="I10" t="s">
-        <v>72</v>
+        <v>177</v>
       </c>
       <c r="J10" t="s">
-        <v>150</v>
+        <v>98</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>70</v>
+        <v>127</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="M10" t="s">
-        <v>101</v>
-      </c>
-      <c r="N10" t="s">
-        <v>176</v>
-      </c>
-      <c r="O10" t="s">
-        <v>177</v>
+        <v>126</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="N10" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="O10" s="1" t="s">
+        <v>130</v>
       </c>
       <c r="P10" t="s">
         <v>65</v>
@@ -1375,7 +1372,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="11" spans="2:17" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:17" ht="128.25" x14ac:dyDescent="0.45">
       <c r="B11" t="s">
         <v>24</v>
       </c>
@@ -1392,28 +1389,28 @@
         <v>5</v>
       </c>
       <c r="H11" t="s">
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="I11" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="J11" t="s">
-        <v>146</v>
+        <v>100</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>159</v>
+        <v>131</v>
       </c>
       <c r="M11" t="s">
-        <v>178</v>
+        <v>134</v>
       </c>
       <c r="N11" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="O11" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="P11" t="s">
         <v>65</v>
@@ -1422,7 +1419,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="2:17" ht="57" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:17" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B12" t="s">
         <v>25</v>
       </c>
@@ -1439,28 +1436,28 @@
         <v>5</v>
       </c>
       <c r="H12" t="s">
-        <v>115</v>
+        <v>77</v>
       </c>
       <c r="I12" t="s">
-        <v>85</v>
+        <v>178</v>
       </c>
       <c r="J12" t="s">
-        <v>147</v>
+        <v>119</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>183</v>
+        <v>137</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>180</v>
+        <v>136</v>
       </c>
       <c r="M12" t="s">
-        <v>82</v>
+        <v>138</v>
       </c>
       <c r="N12" t="s">
-        <v>182</v>
+        <v>140</v>
       </c>
       <c r="O12" t="s">
-        <v>181</v>
+        <v>139</v>
       </c>
       <c r="P12" t="s">
         <v>65</v>
@@ -1486,28 +1483,28 @@
         <v>5</v>
       </c>
       <c r="H13" t="s">
-        <v>116</v>
+        <v>78</v>
       </c>
       <c r="I13" t="s">
-        <v>85</v>
+        <v>72</v>
       </c>
       <c r="J13" t="s">
+        <v>98</v>
+      </c>
+      <c r="K13" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="K13" s="3" t="s">
-        <v>68</v>
-      </c>
       <c r="L13" s="3" t="s">
-        <v>87</v>
+        <v>146</v>
       </c>
       <c r="M13" t="s">
-        <v>88</v>
+        <v>148</v>
       </c>
       <c r="N13" t="s">
-        <v>89</v>
+        <v>149</v>
       </c>
       <c r="O13" t="s">
-        <v>90</v>
+        <v>150</v>
       </c>
       <c r="P13" t="s">
         <v>65</v>
@@ -1533,37 +1530,37 @@
         <v>56</v>
       </c>
       <c r="H14" t="s">
-        <v>117</v>
+        <v>79</v>
       </c>
       <c r="I14" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="J14" t="s">
-        <v>155</v>
+        <v>103</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="L14" s="4" t="s">
-        <v>106</v>
+        <v>142</v>
       </c>
       <c r="M14" t="s">
-        <v>107</v>
+        <v>143</v>
       </c>
       <c r="N14" t="s">
-        <v>108</v>
+        <v>145</v>
       </c>
       <c r="O14" t="s">
-        <v>109</v>
+        <v>144</v>
       </c>
       <c r="P14" t="s">
-        <v>144</v>
+        <v>96</v>
       </c>
       <c r="Q14" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="15" spans="2:17" ht="57" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:17" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B15" t="s">
         <v>57</v>
       </c>
@@ -1580,28 +1577,28 @@
         <v>56</v>
       </c>
       <c r="H15" t="s">
-        <v>118</v>
+        <v>80</v>
       </c>
       <c r="I15" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="J15" t="s">
-        <v>148</v>
+        <v>101</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="L15" s="4" t="s">
-        <v>154</v>
+        <v>162</v>
+      </c>
+      <c r="L15" t="s">
+        <v>160</v>
       </c>
       <c r="M15" t="s">
-        <v>96</v>
+        <v>76</v>
       </c>
       <c r="N15" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="O15" t="s">
-        <v>97</v>
+        <v>161</v>
       </c>
       <c r="P15" t="s">
         <v>65</v>
@@ -1610,7 +1607,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="16" spans="2:17" ht="199.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:17" ht="57" x14ac:dyDescent="0.45">
       <c r="B16" t="s">
         <v>6</v>
       </c>
@@ -1627,28 +1624,28 @@
         <v>18</v>
       </c>
       <c r="H16" t="s">
-        <v>119</v>
+        <v>81</v>
       </c>
       <c r="I16" t="s">
-        <v>124</v>
+        <v>72</v>
       </c>
       <c r="J16" t="s">
-        <v>147</v>
-      </c>
-      <c r="K16" s="3" t="s">
-        <v>67</v>
+        <v>98</v>
+      </c>
+      <c r="K16" t="s">
+        <v>154</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>66</v>
+        <v>158</v>
       </c>
       <c r="M16" t="s">
-        <v>91</v>
+        <v>155</v>
       </c>
       <c r="N16" t="s">
-        <v>92</v>
+        <v>156</v>
       </c>
       <c r="O16" t="s">
-        <v>93</v>
+        <v>157</v>
       </c>
       <c r="P16" t="s">
         <v>65</v>
@@ -1657,63 +1654,63 @@
         <v>65</v>
       </c>
     </row>
-    <row r="17" spans="5:17" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="17" spans="5:17" ht="57" x14ac:dyDescent="0.45">
       <c r="E17" s="1"/>
       <c r="H17" t="s">
-        <v>120</v>
+        <v>82</v>
       </c>
       <c r="I17" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="J17" t="s">
-        <v>147</v>
+        <v>99</v>
       </c>
       <c r="K17" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="L17" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="M17" t="s">
+        <v>153</v>
+      </c>
+      <c r="N17" t="s">
+        <v>152</v>
+      </c>
+      <c r="O17" t="s">
+        <v>151</v>
+      </c>
+      <c r="P17" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="18" spans="5:17" ht="114" x14ac:dyDescent="0.45">
+      <c r="H18" t="s">
+        <v>83</v>
+      </c>
+      <c r="I18" t="s">
+        <v>67</v>
+      </c>
+      <c r="J18" t="s">
+        <v>168</v>
+      </c>
+      <c r="K18" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="L18" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="M18" t="s">
+        <v>166</v>
+      </c>
+      <c r="N18" t="s">
         <v>165</v>
       </c>
-      <c r="L17" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="M17" t="s">
-        <v>110</v>
-      </c>
-      <c r="N17" t="s">
-        <v>111</v>
-      </c>
-      <c r="O17" t="s">
-        <v>112</v>
-      </c>
-      <c r="P17" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q17" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="18" spans="5:17" ht="57" x14ac:dyDescent="0.45">
-      <c r="H18" t="s">
-        <v>121</v>
-      </c>
-      <c r="I18" t="s">
-        <v>85</v>
-      </c>
-      <c r="J18" t="s">
-        <v>147</v>
-      </c>
-      <c r="K18" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="L18" s="4" t="s">
+      <c r="O18" t="s">
         <v>167</v>
-      </c>
-      <c r="M18" t="s">
-        <v>113</v>
-      </c>
-      <c r="N18" t="s">
-        <v>114</v>
-      </c>
-      <c r="O18" t="s">
-        <v>164</v>
       </c>
       <c r="P18" t="s">
         <v>65</v>
@@ -1724,28 +1721,28 @@
     </row>
     <row r="19" spans="5:17" ht="42.75" x14ac:dyDescent="0.45">
       <c r="H19" s="3" t="s">
-        <v>122</v>
+        <v>84</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="J19" t="s">
-        <v>155</v>
+        <v>103</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>129</v>
+        <v>170</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>125</v>
+        <v>86</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>126</v>
+        <v>87</v>
       </c>
       <c r="N19" s="3" t="s">
-        <v>127</v>
+        <v>88</v>
       </c>
       <c r="O19" s="3" t="s">
-        <v>128</v>
+        <v>89</v>
       </c>
       <c r="P19" t="s">
         <v>65</v>
@@ -1756,28 +1753,28 @@
     </row>
     <row r="20" spans="5:17" ht="28.5" x14ac:dyDescent="0.45">
       <c r="H20" s="3" t="s">
-        <v>123</v>
+        <v>85</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="J20" t="s">
-        <v>155</v>
+        <v>103</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>130</v>
+        <v>171</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>131</v>
+        <v>90</v>
       </c>
       <c r="M20" t="s">
-        <v>132</v>
+        <v>91</v>
       </c>
       <c r="N20" t="s">
-        <v>133</v>
+        <v>92</v>
       </c>
       <c r="O20" t="s">
-        <v>134</v>
+        <v>93</v>
       </c>
       <c r="P20" t="s">
         <v>65</v>
@@ -1786,30 +1783,30 @@
         <v>65</v>
       </c>
     </row>
-    <row r="21" spans="5:17" ht="171" x14ac:dyDescent="0.45">
+    <row r="21" spans="5:17" ht="28.5" x14ac:dyDescent="0.45">
       <c r="H21" s="3" t="s">
-        <v>136</v>
+        <v>95</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="J21" t="s">
-        <v>148</v>
+        <v>119</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="L21" s="3" t="s">
-        <v>140</v>
+        <v>172</v>
+      </c>
+      <c r="L21" t="s">
+        <v>174</v>
       </c>
       <c r="M21" t="s">
-        <v>141</v>
+        <v>173</v>
       </c>
       <c r="N21" t="s">
-        <v>142</v>
+        <v>175</v>
       </c>
       <c r="O21" t="s">
-        <v>143</v>
+        <v>176</v>
       </c>
       <c r="P21" t="s">
         <v>65</v>
@@ -1818,69 +1815,28 @@
         <v>65</v>
       </c>
     </row>
-    <row r="22" spans="5:17" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="22" spans="5:17" x14ac:dyDescent="0.45">
       <c r="H22" s="3" t="s">
-        <v>135</v>
+        <v>94</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="J22" t="s">
-        <v>149</v>
-      </c>
-      <c r="K22" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="L22" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="M22" t="s">
-        <v>168</v>
-      </c>
-      <c r="N22" t="s">
-        <v>170</v>
-      </c>
-      <c r="O22" t="s">
-        <v>169</v>
-      </c>
-      <c r="P22" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q22" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="23" spans="5:17" ht="114" x14ac:dyDescent="0.45">
+        <v>67</v>
+      </c>
+      <c r="K22" s="3"/>
+      <c r="L22" s="3"/>
+    </row>
+    <row r="23" spans="5:17" x14ac:dyDescent="0.45">
       <c r="H23" s="3" t="s">
-        <v>158</v>
+        <v>104</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="J23" t="s">
-        <v>148</v>
-      </c>
-      <c r="K23" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="L23" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="M23" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="N23" t="s">
-        <v>99</v>
-      </c>
-      <c r="O23" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="P23" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q23" s="3" t="s">
-        <v>65</v>
-      </c>
+        <v>67</v>
+      </c>
+      <c r="K23" s="3"/>
+      <c r="L23" s="3"/>
+      <c r="M23" s="3"/>
+      <c r="O23" s="3"/>
+      <c r="Q23" s="3"/>
     </row>
     <row r="24" spans="5:17" ht="28.5" x14ac:dyDescent="0.45">
       <c r="H24" s="3"/>
@@ -1889,9 +1845,8 @@
         <v>65</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="L24" s="3"/>
+        <v>66</v>
+      </c>
       <c r="M24" s="3"/>
       <c r="N24" s="3"/>
       <c r="O24" s="3"/>
@@ -1905,7 +1860,7 @@
         <v>65</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="L25" s="3"/>
       <c r="M25" s="3"/>
@@ -1921,7 +1876,7 @@
         <v>65</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="L26" s="3"/>
       <c r="M26" s="3"/>
@@ -1935,7 +1890,7 @@
       <c r="I27" s="3"/>
       <c r="J27" s="3"/>
       <c r="K27" s="3" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="L27" s="3"/>
       <c r="M27" s="3"/>
@@ -1949,7 +1904,7 @@
       <c r="I28" s="3"/>
       <c r="J28" s="3"/>
       <c r="K28" s="3" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="L28" s="3"/>
       <c r="M28" s="3"/>
@@ -1983,19 +1938,29 @@
       <c r="Q30" s="3"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H31:Q33">
-    <cfRule type="expression" dxfId="2" priority="2">
-      <formula>$H31&lt;&gt;""</formula>
+  <conditionalFormatting sqref="H31:Q33 H18:K18 J17:K17 H17 H14:K15 K25:Q26 M24:Q24 K24">
+    <cfRule type="expression" dxfId="5" priority="2">
+      <formula>$H14&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K6">
-    <cfRule type="expression" dxfId="1" priority="1">
+    <cfRule type="expression" dxfId="4" priority="1">
       <formula>$H6&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N6:Q6 H6:J7 L6:L7 P7:Q22 H8:K8 H9:L13 H14:K18 K16:L16 N16:O16 M18:O18 K19:O19 H19:J26 K20:L22 K23 M23 O23 Q23 K24:Q26 H27:Q30">
-    <cfRule type="expression" dxfId="0" priority="3">
+  <conditionalFormatting sqref="N6:Q6 H6:J7 L6:L7 P7:Q22 H8:K8 L16 N16:O16 N18:O18 K19:O19 H19:J26 K20:L20 K23 M23 O23 Q23 H27:Q30 H9:L13 H16:J16 K22:L22 K21">
+    <cfRule type="expression" dxfId="3" priority="3">
       <formula>$H6&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K17">
+    <cfRule type="expression" dxfId="2" priority="5">
+      <formula>$H15&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I16">
+    <cfRule type="expression" dxfId="1" priority="7">
+      <formula>$H17&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
@@ -2007,12 +1972,15 @@
     <hyperlink ref="E12" r:id="rId6" xr:uid="{A248BAB8-B78B-496A-AA69-B3D4947CA9EA}"/>
     <hyperlink ref="E15" r:id="rId7" xr:uid="{EA990D0B-5B76-4CC1-8F1D-936DFD965709}"/>
     <hyperlink ref="E14" r:id="rId8" xr:uid="{22C3A340-0F49-4184-9008-EF45DA2738EA}"/>
+    <hyperlink ref="M10" r:id="rId9" display="mailto:Admin@Excel.net" xr:uid="{8FC561ED-4D1F-495A-B159-FB117F97BB2C}"/>
+    <hyperlink ref="N10" r:id="rId10" display="mailto:Admin@XCEL.net" xr:uid="{4E859147-E45B-43E2-AA1B-BCEE6EFB690B}"/>
+    <hyperlink ref="O10" r:id="rId11" display="mailto:Admin@XCEL.net" xr:uid="{C44698EE-3BC0-44D1-9E94-59F320447E7F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId9"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId12"/>
   <tableParts count="2">
-    <tablePart r:id="rId10"/>
-    <tablePart r:id="rId11"/>
+    <tablePart r:id="rId13"/>
+    <tablePart r:id="rId14"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Lives & Updated Story System
It works
</commit_message>
<xml_diff>
--- a/Assets/Editor/EmailDataExample.xlsx
+++ b/Assets/Editor/EmailDataExample.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joshy\Documents\GitHub\GonePhishing\Assets\Editor\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GameDesign\Programming 3\Final Assignment\Gone Phish\GonePhishing\Assets\Editor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEC38ECB-3312-45FA-90E1-F3FA1AD31FCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A42D2FD-EBA1-48D9-9585-0763F7E79300}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8" yWindow="8" windowWidth="19185" windowHeight="11265" xr2:uid="{3A1DEF22-8015-43E6-8B07-6E12E7B783C7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3A1DEF22-8015-43E6-8B07-6E12E7B783C7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,15 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="180">
   <si>
     <t>Sender</t>
   </si>
@@ -586,6 +583,9 @@
   </si>
   <si>
     <t>Np</t>
+  </si>
+  <si>
+    <t>s1</t>
   </si>
 </sst>
 </file>
@@ -653,16 +653,7 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
-    <dxf>
-      <border>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
+  <dxfs count="5">
     <dxf>
       <border>
         <top style="thin">
@@ -766,9 +757,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -806,7 +797,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -912,7 +903,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1054,7 +1045,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1063,22 +1054,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4422103-5E59-4D36-B01E-BBBBED35EAD4}">
   <dimension ref="B4:Q30"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="4" width="13.59765625" customWidth="1"/>
-    <col min="5" max="5" width="17.59765625" customWidth="1"/>
-    <col min="6" max="6" width="17.3984375" customWidth="1"/>
-    <col min="8" max="10" width="14.59765625" customWidth="1"/>
-    <col min="11" max="11" width="23.59765625" customWidth="1"/>
+    <col min="2" max="4" width="13.5703125" customWidth="1"/>
+    <col min="5" max="5" width="17.5703125" customWidth="1"/>
+    <col min="6" max="6" width="17.42578125" customWidth="1"/>
+    <col min="8" max="10" width="14.5703125" customWidth="1"/>
+    <col min="11" max="11" width="23.5703125" customWidth="1"/>
     <col min="12" max="12" width="48" customWidth="1"/>
-    <col min="13" max="13" width="20.3984375" customWidth="1"/>
-    <col min="14" max="14" width="24.86328125" customWidth="1"/>
-    <col min="15" max="15" width="21.73046875" customWidth="1"/>
-    <col min="16" max="16" width="8.86328125" customWidth="1"/>
-    <col min="17" max="17" width="12.1328125" customWidth="1"/>
+    <col min="13" max="13" width="20.42578125" customWidth="1"/>
+    <col min="14" max="14" width="24.85546875" customWidth="1"/>
+    <col min="15" max="15" width="21.7109375" customWidth="1"/>
+    <col min="16" max="16" width="8.85546875" customWidth="1"/>
+    <col min="17" max="17" width="12.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
         <v>0</v>
       </c>
@@ -1090,7 +1081,7 @@
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
     </row>
-    <row r="5" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>19</v>
       </c>
@@ -1137,7 +1128,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="2:17" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:17" ht="90" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>3</v>
       </c>
@@ -1184,7 +1175,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="7" spans="2:17" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:17" ht="120" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>20</v>
       </c>
@@ -1231,7 +1222,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="2:17" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:17" ht="75" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>44</v>
       </c>
@@ -1278,7 +1269,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="9" spans="2:17" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:17" ht="60" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>51</v>
       </c>
@@ -1325,7 +1316,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="10" spans="2:17" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:17" ht="75" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>47</v>
       </c>
@@ -1366,13 +1357,13 @@
         <v>130</v>
       </c>
       <c r="P10" t="s">
-        <v>65</v>
+        <v>179</v>
       </c>
       <c r="Q10" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="11" spans="2:17" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:17" ht="150" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>24</v>
       </c>
@@ -1419,7 +1410,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="2:17" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:17" ht="45" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>25</v>
       </c>
@@ -1466,7 +1457,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="13" spans="2:17" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:17" ht="135" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>22</v>
       </c>
@@ -1513,7 +1504,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="14" spans="2:17" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:17" ht="120" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>62</v>
       </c>
@@ -1560,7 +1551,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="15" spans="2:17" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:17" ht="30" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>57</v>
       </c>
@@ -1607,7 +1598,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="16" spans="2:17" ht="57" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:17" ht="75" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>6</v>
       </c>
@@ -1654,7 +1645,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="17" spans="5:17" ht="57" x14ac:dyDescent="0.45">
+    <row r="17" spans="5:17" ht="60" x14ac:dyDescent="0.25">
       <c r="E17" s="1"/>
       <c r="H17" t="s">
         <v>82</v>
@@ -1687,7 +1678,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="18" spans="5:17" ht="114" x14ac:dyDescent="0.45">
+    <row r="18" spans="5:17" ht="135" x14ac:dyDescent="0.25">
       <c r="H18" t="s">
         <v>83</v>
       </c>
@@ -1719,7 +1710,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="19" spans="5:17" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="19" spans="5:17" ht="45" x14ac:dyDescent="0.25">
       <c r="H19" s="3" t="s">
         <v>84</v>
       </c>
@@ -1751,7 +1742,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="20" spans="5:17" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="20" spans="5:17" ht="30" x14ac:dyDescent="0.25">
       <c r="H20" s="3" t="s">
         <v>85</v>
       </c>
@@ -1783,7 +1774,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="21" spans="5:17" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="21" spans="5:17" ht="30" x14ac:dyDescent="0.25">
       <c r="H21" s="3" t="s">
         <v>95</v>
       </c>
@@ -1815,7 +1806,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="22" spans="5:17" x14ac:dyDescent="0.45">
+    <row r="22" spans="5:17" x14ac:dyDescent="0.25">
       <c r="H22" s="3" t="s">
         <v>94</v>
       </c>
@@ -1825,7 +1816,7 @@
       <c r="K22" s="3"/>
       <c r="L22" s="3"/>
     </row>
-    <row r="23" spans="5:17" x14ac:dyDescent="0.45">
+    <row r="23" spans="5:17" x14ac:dyDescent="0.25">
       <c r="H23" s="3" t="s">
         <v>104</v>
       </c>
@@ -1838,7 +1829,7 @@
       <c r="O23" s="3"/>
       <c r="Q23" s="3"/>
     </row>
-    <row r="24" spans="5:17" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="24" spans="5:17" ht="30" x14ac:dyDescent="0.25">
       <c r="H24" s="3"/>
       <c r="I24" s="3"/>
       <c r="J24" t="s">
@@ -1853,7 +1844,7 @@
       <c r="P24" s="3"/>
       <c r="Q24" s="3"/>
     </row>
-    <row r="25" spans="5:17" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="25" spans="5:17" ht="30" x14ac:dyDescent="0.25">
       <c r="H25" s="3"/>
       <c r="I25" s="3"/>
       <c r="J25" t="s">
@@ -1869,7 +1860,7 @@
       <c r="P25" s="3"/>
       <c r="Q25" s="3"/>
     </row>
-    <row r="26" spans="5:17" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="26" spans="5:17" ht="30" x14ac:dyDescent="0.25">
       <c r="H26" s="3"/>
       <c r="I26" s="3"/>
       <c r="J26" t="s">
@@ -1885,7 +1876,7 @@
       <c r="P26" s="3"/>
       <c r="Q26" s="3"/>
     </row>
-    <row r="27" spans="5:17" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="27" spans="5:17" ht="30" x14ac:dyDescent="0.25">
       <c r="H27" s="3"/>
       <c r="I27" s="3"/>
       <c r="J27" s="3"/>
@@ -1899,7 +1890,7 @@
       <c r="P27" s="3"/>
       <c r="Q27" s="3"/>
     </row>
-    <row r="28" spans="5:17" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="28" spans="5:17" ht="30" x14ac:dyDescent="0.25">
       <c r="H28" s="3"/>
       <c r="I28" s="3"/>
       <c r="J28" s="3"/>
@@ -1913,7 +1904,7 @@
       <c r="P28" s="3"/>
       <c r="Q28" s="3"/>
     </row>
-    <row r="29" spans="5:17" x14ac:dyDescent="0.45">
+    <row r="29" spans="5:17" x14ac:dyDescent="0.25">
       <c r="H29" s="3"/>
       <c r="I29" s="3"/>
       <c r="J29" s="3"/>
@@ -1925,7 +1916,7 @@
       <c r="P29" s="3"/>
       <c r="Q29" s="3"/>
     </row>
-    <row r="30" spans="5:17" x14ac:dyDescent="0.45">
+    <row r="30" spans="5:17" x14ac:dyDescent="0.25">
       <c r="H30" s="3"/>
       <c r="I30" s="3"/>
       <c r="J30" s="3"/>
@@ -1938,29 +1929,29 @@
       <c r="Q30" s="3"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H31:Q33 H18:K18 J17:K17 H17 H14:K15 K25:Q26 M24:Q24 K24">
-    <cfRule type="expression" dxfId="5" priority="2">
+  <conditionalFormatting sqref="H14:K15 H17 J17:K17 H18:K18 K23:K24 M24:Q24 K25:Q26 H31:Q33">
+    <cfRule type="expression" dxfId="4" priority="2">
       <formula>$H14&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K6">
-    <cfRule type="expression" dxfId="4" priority="1">
-      <formula>$H6&lt;&gt;""</formula>
+  <conditionalFormatting sqref="I16">
+    <cfRule type="expression" dxfId="3" priority="7">
+      <formula>$H17&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N6:Q6 H6:J7 L6:L7 P7:Q22 H8:K8 L16 N16:O16 N18:O18 K19:O19 H19:J26 K20:L20 K23 M23 O23 Q23 H27:Q30 H9:L13 H16:J16 K22:L22 K21">
-    <cfRule type="expression" dxfId="3" priority="3">
+  <conditionalFormatting sqref="K6">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>$H6&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K17">
-    <cfRule type="expression" dxfId="2" priority="5">
+    <cfRule type="expression" dxfId="1" priority="5">
       <formula>$H15&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I16">
-    <cfRule type="expression" dxfId="1" priority="7">
-      <formula>$H17&lt;&gt;""</formula>
+  <conditionalFormatting sqref="N6:Q6 H6:J7 L6:L7 P7:Q22 H8:K8 H9:L13 H16:J16 L16 N16:O16 N18:O18 K19:O19 H19:J26 K20:L20 K21 K22:L22 M23 O23 Q23 H27:Q30">
+    <cfRule type="expression" dxfId="0" priority="3">
+      <formula>$H6&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>

</xml_diff>